<commit_message>
Touchbistro stable with .bat for weekly reporting
</commit_message>
<xml_diff>
--- a/checker_template.xlsx
+++ b/checker_template.xlsx
@@ -477,7 +477,7 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="58">
+  <cellXfs count="62">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="1" fontId="2" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -585,6 +585,18 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="1" fontId="0" fillId="5" borderId="30" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="5" fillId="0" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="5" fillId="0" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="5" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="5" fillId="0" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -953,12 +965,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X82"/>
+  <dimension ref="A1:AB82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9.85546875" customWidth="1" min="1" max="1"/>
     <col width="42.85546875" customWidth="1" min="2" max="2"/>
     <col width="9.85546875" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="19" max="19"/>
+    <col width="10" customWidth="1" min="20" max="20"/>
+    <col width="12" customWidth="1" min="21" max="21"/>
+    <col width="10" customWidth="1" min="22" max="22"/>
   </cols>
   <sheetData>
     <row r="1" ht="15.75" customHeight="1" thickBot="1">
@@ -989,7 +1005,11 @@
       <c r="U1" s="41" t="n"/>
       <c r="V1" s="41" t="n"/>
       <c r="W1" s="41" t="n"/>
-      <c r="X1" s="42" t="n"/>
+      <c r="X1" s="41" t="n"/>
+      <c r="Y1" s="41" t="n"/>
+      <c r="Z1" s="41" t="n"/>
+      <c r="AA1" s="41" t="n"/>
+      <c r="AB1" s="42" t="n"/>
     </row>
     <row r="2" ht="15" customHeight="1" thickBot="1">
       <c r="A2" s="43" t="n"/>
@@ -1015,7 +1035,11 @@
       <c r="U2" s="44" t="n"/>
       <c r="V2" s="44" t="n"/>
       <c r="W2" s="44" t="n"/>
-      <c r="X2" s="45" t="n"/>
+      <c r="X2" s="44" t="n"/>
+      <c r="Y2" s="44" t="n"/>
+      <c r="Z2" s="44" t="n"/>
+      <c r="AA2" s="44" t="n"/>
+      <c r="AB2" s="45" t="n"/>
     </row>
     <row r="3" ht="15" customHeight="1" thickBot="1">
       <c r="A3" s="1" t="n"/>
@@ -1106,30 +1130,50 @@
       </c>
       <c r="S3" s="3" t="inlineStr">
         <is>
+          <t>oshawa</t>
+        </is>
+      </c>
+      <c r="T3" s="3" t="inlineStr">
+        <is>
+          <t>percentage</t>
+        </is>
+      </c>
+      <c r="U3" s="3" t="inlineStr">
+        <is>
+          <t>milton</t>
+        </is>
+      </c>
+      <c r="V3" s="3" t="inlineStr">
+        <is>
+          <t>percentage</t>
+        </is>
+      </c>
+      <c r="W3" s="3" t="inlineStr">
+        <is>
           <t>food court</t>
         </is>
       </c>
-      <c r="T3" s="4" t="inlineStr">
+      <c r="X3" s="4" t="inlineStr">
         <is>
           <t>percentage</t>
         </is>
       </c>
-      <c r="U3" s="5" t="inlineStr">
+      <c r="Y3" s="5" t="inlineStr">
         <is>
           <t>kabab wala</t>
         </is>
       </c>
-      <c r="V3" s="6" t="inlineStr">
+      <c r="Z3" s="6" t="inlineStr">
         <is>
           <t>percentage</t>
         </is>
       </c>
-      <c r="W3" s="7" t="inlineStr">
+      <c r="AA3" s="7" t="inlineStr">
         <is>
           <t>kababwala Q St</t>
         </is>
       </c>
-      <c r="X3" s="6" t="inlineStr">
+      <c r="AB3" s="6" t="inlineStr">
         <is>
           <t>percentage</t>
         </is>
@@ -1186,20 +1230,30 @@
         <v/>
       </c>
       <c r="R4" s="10" t="n"/>
-      <c r="S4" s="11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="T4" s="9" t="n"/>
-      <c r="U4" s="9" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="V4" s="12" t="n"/>
-      <c r="W4" s="12" t="n"/>
-      <c r="X4" s="13" t="n"/>
+      <c r="S4" s="58">
+        <f>IFERROR(SUMIF(Oshawa!$A:$A, B4, Oshawa!$F:$F), 0)</f>
+        <v/>
+      </c>
+      <c r="T4" s="58" t="n"/>
+      <c r="U4" s="58">
+        <f>IFERROR(SUMIF(Milton!$A:$A, B4, Milton!$F:$F), 0)</f>
+        <v/>
+      </c>
+      <c r="V4" s="58" t="n"/>
+      <c r="W4" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="X4" s="9" t="n"/>
+      <c r="Y4" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Z4" s="12" t="n"/>
+      <c r="AA4" s="12" t="n"/>
+      <c r="AB4" s="13" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="55" t="n"/>
@@ -1248,20 +1302,30 @@
         <v/>
       </c>
       <c r="R5" s="10" t="n"/>
-      <c r="S5" s="11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="T5" s="9" t="n"/>
-      <c r="U5" s="9" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="V5" s="12" t="n"/>
-      <c r="W5" s="12" t="n"/>
-      <c r="X5" s="13" t="n"/>
+      <c r="S5" s="58">
+        <f>IFERROR(SUMIF(Oshawa!$A:$A, B5, Oshawa!$F:$F), 0)</f>
+        <v/>
+      </c>
+      <c r="T5" s="58" t="n"/>
+      <c r="U5" s="58">
+        <f>IFERROR(SUMIF(Milton!$A:$A, B5, Milton!$F:$F), 0)</f>
+        <v/>
+      </c>
+      <c r="V5" s="58" t="n"/>
+      <c r="W5" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="X5" s="9" t="n"/>
+      <c r="Y5" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Z5" s="12" t="n"/>
+      <c r="AA5" s="12" t="n"/>
+      <c r="AB5" s="13" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="55" t="n"/>
@@ -1310,20 +1374,30 @@
         <v/>
       </c>
       <c r="R6" s="10" t="n"/>
-      <c r="S6" s="11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="T6" s="9" t="n"/>
-      <c r="U6" s="9" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="V6" s="12" t="n"/>
-      <c r="W6" s="12" t="n"/>
-      <c r="X6" s="13" t="n"/>
+      <c r="S6" s="58">
+        <f>IFERROR(SUMIF(Oshawa!$A:$A, B6, Oshawa!$F:$F), 0)</f>
+        <v/>
+      </c>
+      <c r="T6" s="58" t="n"/>
+      <c r="U6" s="58">
+        <f>IFERROR(SUMIF(Milton!$A:$A, B6, Milton!$F:$F), 0)</f>
+        <v/>
+      </c>
+      <c r="V6" s="58" t="n"/>
+      <c r="W6" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="X6" s="9" t="n"/>
+      <c r="Y6" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Z6" s="12" t="n"/>
+      <c r="AA6" s="12" t="n"/>
+      <c r="AB6" s="13" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="55" t="n"/>
@@ -1372,20 +1446,30 @@
         <v/>
       </c>
       <c r="R7" s="10" t="n"/>
-      <c r="S7" s="11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="T7" s="9" t="n"/>
-      <c r="U7" s="9" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="V7" s="12" t="n"/>
-      <c r="W7" s="12" t="n"/>
-      <c r="X7" s="13" t="n"/>
+      <c r="S7" s="59">
+        <f>IFERROR(SUMIF(Oshawa!$A:$A, B7, Oshawa!$F:$F), 0)</f>
+        <v/>
+      </c>
+      <c r="T7" s="59" t="n"/>
+      <c r="U7" s="59">
+        <f>IFERROR(SUMIF(Milton!$A:$A, B7, Milton!$F:$F), 0)</f>
+        <v/>
+      </c>
+      <c r="V7" s="59" t="n"/>
+      <c r="W7" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="X7" s="9" t="n"/>
+      <c r="Y7" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Z7" s="12" t="n"/>
+      <c r="AA7" s="12" t="n"/>
+      <c r="AB7" s="13" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="55" t="n"/>
@@ -1434,20 +1518,30 @@
         <v/>
       </c>
       <c r="R8" s="10" t="n"/>
-      <c r="S8" s="11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="T8" s="9" t="n"/>
-      <c r="U8" s="9" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="V8" s="12" t="n"/>
-      <c r="W8" s="12" t="n"/>
-      <c r="X8" s="13" t="n"/>
+      <c r="S8" s="59">
+        <f>IFERROR(SUMIF(Oshawa!$A:$A, B8, Oshawa!$F:$F), 0)</f>
+        <v/>
+      </c>
+      <c r="T8" s="59" t="n"/>
+      <c r="U8" s="59">
+        <f>IFERROR(SUMIF(Milton!$A:$A, B8, Milton!$F:$F), 0)</f>
+        <v/>
+      </c>
+      <c r="V8" s="59" t="n"/>
+      <c r="W8" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="X8" s="9" t="n"/>
+      <c r="Y8" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Z8" s="12" t="n"/>
+      <c r="AA8" s="12" t="n"/>
+      <c r="AB8" s="13" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="55" t="n"/>
@@ -1496,12 +1590,22 @@
         <v/>
       </c>
       <c r="R9" s="10" t="n"/>
-      <c r="S9" s="11" t="n"/>
-      <c r="T9" s="9" t="n"/>
-      <c r="U9" s="9" t="n"/>
-      <c r="V9" s="12" t="n"/>
-      <c r="W9" s="12" t="n"/>
-      <c r="X9" s="13" t="n"/>
+      <c r="S9" s="59">
+        <f>IFERROR(SUMIF(Oshawa!$A:$A, B9, Oshawa!$F:$F), 0)</f>
+        <v/>
+      </c>
+      <c r="T9" s="59" t="n"/>
+      <c r="U9" s="59">
+        <f>IFERROR(SUMIF(Milton!$A:$A, B9, Milton!$F:$F), 0)</f>
+        <v/>
+      </c>
+      <c r="V9" s="59" t="n"/>
+      <c r="W9" s="11" t="n"/>
+      <c r="X9" s="9" t="n"/>
+      <c r="Y9" s="9" t="n"/>
+      <c r="Z9" s="12" t="n"/>
+      <c r="AA9" s="12" t="n"/>
+      <c r="AB9" s="13" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="55" t="n"/>
@@ -1550,12 +1654,22 @@
         <v/>
       </c>
       <c r="R10" s="10" t="n"/>
-      <c r="S10" s="11" t="n"/>
-      <c r="T10" s="9" t="n"/>
-      <c r="U10" s="9" t="n"/>
-      <c r="V10" s="12" t="n"/>
-      <c r="W10" s="12" t="n"/>
-      <c r="X10" s="13" t="n"/>
+      <c r="S10" s="59">
+        <f>IFERROR(SUMIF(Oshawa!$A:$A, B10, Oshawa!$F:$F), 0)</f>
+        <v/>
+      </c>
+      <c r="T10" s="59" t="n"/>
+      <c r="U10" s="59">
+        <f>IFERROR(SUMIF(Milton!$A:$A, B10, Milton!$F:$F), 0)</f>
+        <v/>
+      </c>
+      <c r="V10" s="59" t="n"/>
+      <c r="W10" s="11" t="n"/>
+      <c r="X10" s="9" t="n"/>
+      <c r="Y10" s="9" t="n"/>
+      <c r="Z10" s="12" t="n"/>
+      <c r="AA10" s="12" t="n"/>
+      <c r="AB10" s="13" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="55" t="n"/>
@@ -1604,12 +1718,22 @@
         <v/>
       </c>
       <c r="R11" s="10" t="n"/>
-      <c r="S11" s="11" t="n"/>
-      <c r="T11" s="9" t="n"/>
-      <c r="U11" s="9" t="n"/>
-      <c r="V11" s="12" t="n"/>
-      <c r="W11" s="12" t="n"/>
-      <c r="X11" s="13" t="n"/>
+      <c r="S11" s="59">
+        <f>IFERROR(SUMIF(Oshawa!$A:$A, B11, Oshawa!$F:$F), 0)</f>
+        <v/>
+      </c>
+      <c r="T11" s="59" t="n"/>
+      <c r="U11" s="59">
+        <f>IFERROR(SUMIF(Milton!$A:$A, B11, Milton!$F:$F), 0)</f>
+        <v/>
+      </c>
+      <c r="V11" s="59" t="n"/>
+      <c r="W11" s="11" t="n"/>
+      <c r="X11" s="9" t="n"/>
+      <c r="Y11" s="9" t="n"/>
+      <c r="Z11" s="12" t="n"/>
+      <c r="AA11" s="12" t="n"/>
+      <c r="AB11" s="13" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="55" t="n"/>
@@ -1658,12 +1782,22 @@
         <v/>
       </c>
       <c r="R12" s="10" t="n"/>
-      <c r="S12" s="11" t="n"/>
-      <c r="T12" s="9" t="n"/>
-      <c r="U12" s="9" t="n"/>
-      <c r="V12" s="12" t="n"/>
-      <c r="W12" s="12" t="n"/>
-      <c r="X12" s="13" t="n"/>
+      <c r="S12" s="59">
+        <f>IFERROR(SUMIF(Oshawa!$A:$A, B12, Oshawa!$F:$F), 0)</f>
+        <v/>
+      </c>
+      <c r="T12" s="59" t="n"/>
+      <c r="U12" s="59">
+        <f>IFERROR(SUMIF(Milton!$A:$A, B12, Milton!$F:$F), 0)</f>
+        <v/>
+      </c>
+      <c r="V12" s="59" t="n"/>
+      <c r="W12" s="11" t="n"/>
+      <c r="X12" s="9" t="n"/>
+      <c r="Y12" s="9" t="n"/>
+      <c r="Z12" s="12" t="n"/>
+      <c r="AA12" s="12" t="n"/>
+      <c r="AB12" s="13" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="55" t="n"/>
@@ -1712,12 +1846,22 @@
         <v/>
       </c>
       <c r="R13" s="10" t="n"/>
-      <c r="S13" s="11" t="n"/>
-      <c r="T13" s="9" t="n"/>
-      <c r="U13" s="9" t="n"/>
-      <c r="V13" s="12" t="n"/>
-      <c r="W13" s="12" t="n"/>
-      <c r="X13" s="13" t="n"/>
+      <c r="S13" s="59">
+        <f>IFERROR(SUMIF(Oshawa!$A:$A, B13, Oshawa!$F:$F), 0)</f>
+        <v/>
+      </c>
+      <c r="T13" s="59" t="n"/>
+      <c r="U13" s="59">
+        <f>IFERROR(SUMIF(Milton!$A:$A, B13, Milton!$F:$F), 0)</f>
+        <v/>
+      </c>
+      <c r="V13" s="59" t="n"/>
+      <c r="W13" s="11" t="n"/>
+      <c r="X13" s="9" t="n"/>
+      <c r="Y13" s="9" t="n"/>
+      <c r="Z13" s="12" t="n"/>
+      <c r="AA13" s="12" t="n"/>
+      <c r="AB13" s="13" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="55" t="n"/>
@@ -1766,12 +1910,22 @@
         <v/>
       </c>
       <c r="R14" s="10" t="n"/>
-      <c r="S14" s="11" t="n"/>
-      <c r="T14" s="9" t="n"/>
-      <c r="U14" s="9" t="n"/>
-      <c r="V14" s="12" t="n"/>
-      <c r="W14" s="12" t="n"/>
-      <c r="X14" s="13" t="n"/>
+      <c r="S14" s="59">
+        <f>IFERROR(SUMIF(Oshawa!$A:$A, B14, Oshawa!$F:$F), 0)</f>
+        <v/>
+      </c>
+      <c r="T14" s="59" t="n"/>
+      <c r="U14" s="59">
+        <f>IFERROR(SUMIF(Milton!$A:$A, B14, Milton!$F:$F), 0)</f>
+        <v/>
+      </c>
+      <c r="V14" s="59" t="n"/>
+      <c r="W14" s="11" t="n"/>
+      <c r="X14" s="9" t="n"/>
+      <c r="Y14" s="9" t="n"/>
+      <c r="Z14" s="12" t="n"/>
+      <c r="AA14" s="12" t="n"/>
+      <c r="AB14" s="13" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="55" t="n"/>
@@ -1820,12 +1974,22 @@
         <v/>
       </c>
       <c r="R15" s="10" t="n"/>
-      <c r="S15" s="11" t="n"/>
-      <c r="T15" s="9" t="n"/>
-      <c r="U15" s="9" t="n"/>
-      <c r="V15" s="12" t="n"/>
-      <c r="W15" s="12" t="n"/>
-      <c r="X15" s="13" t="n"/>
+      <c r="S15" s="59">
+        <f>IFERROR(SUMIF(Oshawa!$A:$A, B15, Oshawa!$F:$F), 0)</f>
+        <v/>
+      </c>
+      <c r="T15" s="59" t="n"/>
+      <c r="U15" s="59">
+        <f>IFERROR(SUMIF(Milton!$A:$A, B15, Milton!$F:$F), 0)</f>
+        <v/>
+      </c>
+      <c r="V15" s="59" t="n"/>
+      <c r="W15" s="11" t="n"/>
+      <c r="X15" s="9" t="n"/>
+      <c r="Y15" s="9" t="n"/>
+      <c r="Z15" s="12" t="n"/>
+      <c r="AA15" s="12" t="n"/>
+      <c r="AB15" s="13" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="55" t="n"/>
@@ -1874,12 +2038,22 @@
         <v/>
       </c>
       <c r="R16" s="10" t="n"/>
-      <c r="S16" s="11" t="n"/>
-      <c r="T16" s="9" t="n"/>
-      <c r="U16" s="9" t="n"/>
-      <c r="V16" s="12" t="n"/>
-      <c r="W16" s="12" t="n"/>
-      <c r="X16" s="13" t="n"/>
+      <c r="S16" s="59">
+        <f>IFERROR(SUMIF(Oshawa!$A:$A, B16, Oshawa!$F:$F), 0)</f>
+        <v/>
+      </c>
+      <c r="T16" s="59" t="n"/>
+      <c r="U16" s="59">
+        <f>IFERROR(SUMIF(Milton!$A:$A, B16, Milton!$F:$F), 0)</f>
+        <v/>
+      </c>
+      <c r="V16" s="59" t="n"/>
+      <c r="W16" s="11" t="n"/>
+      <c r="X16" s="9" t="n"/>
+      <c r="Y16" s="9" t="n"/>
+      <c r="Z16" s="12" t="n"/>
+      <c r="AA16" s="12" t="n"/>
+      <c r="AB16" s="13" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="55" t="n"/>
@@ -1928,12 +2102,22 @@
         <v/>
       </c>
       <c r="R17" s="10" t="n"/>
-      <c r="S17" s="11" t="n"/>
-      <c r="T17" s="9" t="n"/>
-      <c r="U17" s="9" t="n"/>
-      <c r="V17" s="12" t="n"/>
-      <c r="W17" s="12" t="n"/>
-      <c r="X17" s="13" t="n"/>
+      <c r="S17" s="59">
+        <f>IFERROR(SUMIF(Oshawa!$A:$A, B17, Oshawa!$F:$F), 0)</f>
+        <v/>
+      </c>
+      <c r="T17" s="59" t="n"/>
+      <c r="U17" s="59">
+        <f>IFERROR(SUMIF(Milton!$A:$A, B17, Milton!$F:$F), 0)</f>
+        <v/>
+      </c>
+      <c r="V17" s="59" t="n"/>
+      <c r="W17" s="11" t="n"/>
+      <c r="X17" s="9" t="n"/>
+      <c r="Y17" s="9" t="n"/>
+      <c r="Z17" s="12" t="n"/>
+      <c r="AA17" s="12" t="n"/>
+      <c r="AB17" s="13" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="55" t="n"/>
@@ -1982,12 +2166,22 @@
         <v/>
       </c>
       <c r="R18" s="10" t="n"/>
-      <c r="S18" s="11" t="n"/>
-      <c r="T18" s="9" t="n"/>
-      <c r="U18" s="9" t="n"/>
-      <c r="V18" s="12" t="n"/>
-      <c r="W18" s="12" t="n"/>
-      <c r="X18" s="13" t="n"/>
+      <c r="S18" s="59">
+        <f>IFERROR(SUMIF(Oshawa!$A:$A, B18, Oshawa!$F:$F), 0)</f>
+        <v/>
+      </c>
+      <c r="T18" s="59" t="n"/>
+      <c r="U18" s="59">
+        <f>IFERROR(SUMIF(Milton!$A:$A, B18, Milton!$F:$F), 0)</f>
+        <v/>
+      </c>
+      <c r="V18" s="59" t="n"/>
+      <c r="W18" s="11" t="n"/>
+      <c r="X18" s="9" t="n"/>
+      <c r="Y18" s="9" t="n"/>
+      <c r="Z18" s="12" t="n"/>
+      <c r="AA18" s="12" t="n"/>
+      <c r="AB18" s="13" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="55" t="n"/>
@@ -2036,12 +2230,22 @@
         <v/>
       </c>
       <c r="R19" s="10" t="n"/>
-      <c r="S19" s="11" t="n"/>
-      <c r="T19" s="9" t="n"/>
-      <c r="U19" s="9" t="n"/>
-      <c r="V19" s="12" t="n"/>
-      <c r="W19" s="12" t="n"/>
-      <c r="X19" s="13" t="n"/>
+      <c r="S19" s="59">
+        <f>IFERROR(SUMIF(Oshawa!$A:$A, B19, Oshawa!$F:$F), 0)</f>
+        <v/>
+      </c>
+      <c r="T19" s="59" t="n"/>
+      <c r="U19" s="59">
+        <f>IFERROR(SUMIF(Milton!$A:$A, B19, Milton!$F:$F), 0)</f>
+        <v/>
+      </c>
+      <c r="V19" s="59" t="n"/>
+      <c r="W19" s="11" t="n"/>
+      <c r="X19" s="9" t="n"/>
+      <c r="Y19" s="9" t="n"/>
+      <c r="Z19" s="12" t="n"/>
+      <c r="AA19" s="12" t="n"/>
+      <c r="AB19" s="13" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="55" t="n"/>
@@ -2090,12 +2294,22 @@
         <v/>
       </c>
       <c r="R20" s="10" t="n"/>
-      <c r="S20" s="11" t="n"/>
-      <c r="T20" s="9" t="n"/>
-      <c r="U20" s="9" t="n"/>
-      <c r="V20" s="12" t="n"/>
-      <c r="W20" s="12" t="n"/>
-      <c r="X20" s="13" t="n"/>
+      <c r="S20" s="59">
+        <f>IFERROR(SUMIF(Oshawa!$A:$A, B20, Oshawa!$F:$F), 0)</f>
+        <v/>
+      </c>
+      <c r="T20" s="59" t="n"/>
+      <c r="U20" s="59">
+        <f>IFERROR(SUMIF(Milton!$A:$A, B20, Milton!$F:$F), 0)</f>
+        <v/>
+      </c>
+      <c r="V20" s="59" t="n"/>
+      <c r="W20" s="11" t="n"/>
+      <c r="X20" s="9" t="n"/>
+      <c r="Y20" s="9" t="n"/>
+      <c r="Z20" s="12" t="n"/>
+      <c r="AA20" s="12" t="n"/>
+      <c r="AB20" s="13" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="55" t="n"/>
@@ -2144,12 +2358,22 @@
         <v/>
       </c>
       <c r="R21" s="10" t="n"/>
-      <c r="S21" s="11" t="n"/>
-      <c r="T21" s="9" t="n"/>
-      <c r="U21" s="9" t="n"/>
-      <c r="V21" s="12" t="n"/>
-      <c r="W21" s="12" t="n"/>
-      <c r="X21" s="13" t="n"/>
+      <c r="S21" s="59">
+        <f>IFERROR(SUMIF(Oshawa!$A:$A, B21, Oshawa!$F:$F), 0)</f>
+        <v/>
+      </c>
+      <c r="T21" s="59" t="n"/>
+      <c r="U21" s="59">
+        <f>IFERROR(SUMIF(Milton!$A:$A, B21, Milton!$F:$F), 0)</f>
+        <v/>
+      </c>
+      <c r="V21" s="59" t="n"/>
+      <c r="W21" s="11" t="n"/>
+      <c r="X21" s="9" t="n"/>
+      <c r="Y21" s="9" t="n"/>
+      <c r="Z21" s="12" t="n"/>
+      <c r="AA21" s="12" t="n"/>
+      <c r="AB21" s="13" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="55" t="n"/>
@@ -2198,12 +2422,22 @@
         <v/>
       </c>
       <c r="R22" s="10" t="n"/>
-      <c r="S22" s="11" t="n"/>
-      <c r="T22" s="9" t="n"/>
-      <c r="U22" s="9" t="n"/>
-      <c r="V22" s="12" t="n"/>
-      <c r="W22" s="12" t="n"/>
-      <c r="X22" s="13" t="n"/>
+      <c r="S22" s="59">
+        <f>IFERROR(SUMIF(Oshawa!$A:$A, B22, Oshawa!$F:$F), 0)</f>
+        <v/>
+      </c>
+      <c r="T22" s="59" t="n"/>
+      <c r="U22" s="59">
+        <f>IFERROR(SUMIF(Milton!$A:$A, B22, Milton!$F:$F), 0)</f>
+        <v/>
+      </c>
+      <c r="V22" s="59" t="n"/>
+      <c r="W22" s="11" t="n"/>
+      <c r="X22" s="9" t="n"/>
+      <c r="Y22" s="9" t="n"/>
+      <c r="Z22" s="12" t="n"/>
+      <c r="AA22" s="12" t="n"/>
+      <c r="AB22" s="13" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="55" t="n"/>
@@ -2252,12 +2486,22 @@
         <v/>
       </c>
       <c r="R23" s="10" t="n"/>
-      <c r="S23" s="11" t="n"/>
-      <c r="T23" s="9" t="n"/>
-      <c r="U23" s="9" t="n"/>
-      <c r="V23" s="12" t="n"/>
-      <c r="W23" s="12" t="n"/>
-      <c r="X23" s="13" t="n"/>
+      <c r="S23" s="59">
+        <f>IFERROR(SUMIF(Oshawa!$A:$A, B23, Oshawa!$F:$F), 0)</f>
+        <v/>
+      </c>
+      <c r="T23" s="59" t="n"/>
+      <c r="U23" s="59">
+        <f>IFERROR(SUMIF(Milton!$A:$A, B23, Milton!$F:$F), 0)</f>
+        <v/>
+      </c>
+      <c r="V23" s="59" t="n"/>
+      <c r="W23" s="11" t="n"/>
+      <c r="X23" s="9" t="n"/>
+      <c r="Y23" s="9" t="n"/>
+      <c r="Z23" s="12" t="n"/>
+      <c r="AA23" s="12" t="n"/>
+      <c r="AB23" s="13" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="55" t="n"/>
@@ -2306,12 +2550,22 @@
         <v/>
       </c>
       <c r="R24" s="10" t="n"/>
-      <c r="S24" s="11" t="n"/>
-      <c r="T24" s="9" t="n"/>
-      <c r="U24" s="9" t="n"/>
-      <c r="V24" s="12" t="n"/>
-      <c r="W24" s="12" t="n"/>
-      <c r="X24" s="13" t="n"/>
+      <c r="S24" s="59">
+        <f>IFERROR(SUMIF(Oshawa!$A:$A, B24, Oshawa!$F:$F), 0)</f>
+        <v/>
+      </c>
+      <c r="T24" s="59" t="n"/>
+      <c r="U24" s="59">
+        <f>IFERROR(SUMIF(Milton!$A:$A, B24, Milton!$F:$F), 0)</f>
+        <v/>
+      </c>
+      <c r="V24" s="59" t="n"/>
+      <c r="W24" s="11" t="n"/>
+      <c r="X24" s="9" t="n"/>
+      <c r="Y24" s="9" t="n"/>
+      <c r="Z24" s="12" t="n"/>
+      <c r="AA24" s="12" t="n"/>
+      <c r="AB24" s="13" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="55" t="n"/>
@@ -2360,12 +2614,22 @@
         <v/>
       </c>
       <c r="R25" s="10" t="n"/>
-      <c r="S25" s="11" t="n"/>
-      <c r="T25" s="9" t="n"/>
-      <c r="U25" s="9" t="n"/>
-      <c r="V25" s="12" t="n"/>
-      <c r="W25" s="12" t="n"/>
-      <c r="X25" s="13" t="n"/>
+      <c r="S25" s="59">
+        <f>IFERROR(SUMIF(Oshawa!$A:$A, B25, Oshawa!$F:$F), 0)</f>
+        <v/>
+      </c>
+      <c r="T25" s="59" t="n"/>
+      <c r="U25" s="59">
+        <f>IFERROR(SUMIF(Milton!$A:$A, B25, Milton!$F:$F), 0)</f>
+        <v/>
+      </c>
+      <c r="V25" s="59" t="n"/>
+      <c r="W25" s="11" t="n"/>
+      <c r="X25" s="9" t="n"/>
+      <c r="Y25" s="9" t="n"/>
+      <c r="Z25" s="12" t="n"/>
+      <c r="AA25" s="12" t="n"/>
+      <c r="AB25" s="13" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="55" t="n"/>
@@ -2414,12 +2678,22 @@
         <v/>
       </c>
       <c r="R26" s="10" t="n"/>
-      <c r="S26" s="11" t="n"/>
-      <c r="T26" s="9" t="n"/>
-      <c r="U26" s="9" t="n"/>
-      <c r="V26" s="12" t="n"/>
-      <c r="W26" s="12" t="n"/>
-      <c r="X26" s="13" t="n"/>
+      <c r="S26" s="59">
+        <f>IFERROR(SUMIF(Oshawa!$A:$A, B26, Oshawa!$F:$F), 0)</f>
+        <v/>
+      </c>
+      <c r="T26" s="59" t="n"/>
+      <c r="U26" s="59">
+        <f>IFERROR(SUMIF(Milton!$A:$A, B26, Milton!$F:$F), 0)</f>
+        <v/>
+      </c>
+      <c r="V26" s="59" t="n"/>
+      <c r="W26" s="11" t="n"/>
+      <c r="X26" s="9" t="n"/>
+      <c r="Y26" s="9" t="n"/>
+      <c r="Z26" s="12" t="n"/>
+      <c r="AA26" s="12" t="n"/>
+      <c r="AB26" s="13" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="55" t="n"/>
@@ -2468,12 +2742,22 @@
         <v/>
       </c>
       <c r="R27" s="10" t="n"/>
-      <c r="S27" s="11" t="n"/>
-      <c r="T27" s="9" t="n"/>
-      <c r="U27" s="9" t="n"/>
-      <c r="V27" s="12" t="n"/>
-      <c r="W27" s="12" t="n"/>
-      <c r="X27" s="13" t="n"/>
+      <c r="S27" s="59">
+        <f>IFERROR(SUMIF(Oshawa!$A:$A, B27, Oshawa!$F:$F), 0)</f>
+        <v/>
+      </c>
+      <c r="T27" s="59" t="n"/>
+      <c r="U27" s="59">
+        <f>IFERROR(SUMIF(Milton!$A:$A, B27, Milton!$F:$F), 0)</f>
+        <v/>
+      </c>
+      <c r="V27" s="59" t="n"/>
+      <c r="W27" s="11" t="n"/>
+      <c r="X27" s="9" t="n"/>
+      <c r="Y27" s="9" t="n"/>
+      <c r="Z27" s="12" t="n"/>
+      <c r="AA27" s="12" t="n"/>
+      <c r="AB27" s="13" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="55" t="n"/>
@@ -2522,12 +2806,22 @@
         <v/>
       </c>
       <c r="R28" s="10" t="n"/>
-      <c r="S28" s="11" t="n"/>
-      <c r="T28" s="9" t="n"/>
-      <c r="U28" s="9" t="n"/>
-      <c r="V28" s="12" t="n"/>
-      <c r="W28" s="12" t="n"/>
-      <c r="X28" s="13" t="n"/>
+      <c r="S28" s="59">
+        <f>IFERROR(SUMIF(Oshawa!$A:$A, B28, Oshawa!$F:$F), 0)</f>
+        <v/>
+      </c>
+      <c r="T28" s="59" t="n"/>
+      <c r="U28" s="59">
+        <f>IFERROR(SUMIF(Milton!$A:$A, B28, Milton!$F:$F), 0)</f>
+        <v/>
+      </c>
+      <c r="V28" s="59" t="n"/>
+      <c r="W28" s="11" t="n"/>
+      <c r="X28" s="9" t="n"/>
+      <c r="Y28" s="9" t="n"/>
+      <c r="Z28" s="12" t="n"/>
+      <c r="AA28" s="12" t="n"/>
+      <c r="AB28" s="13" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="55" t="n"/>
@@ -2576,12 +2870,22 @@
         <v/>
       </c>
       <c r="R29" s="21" t="n"/>
-      <c r="S29" s="9" t="n"/>
-      <c r="T29" s="21" t="n"/>
-      <c r="U29" s="9" t="n"/>
-      <c r="V29" s="21" t="n"/>
+      <c r="S29" s="59">
+        <f>IFERROR(SUMIF(Oshawa!$A:$A, B29, Oshawa!$F:$F), 0)</f>
+        <v/>
+      </c>
+      <c r="T29" s="59" t="n"/>
+      <c r="U29" s="59">
+        <f>IFERROR(SUMIF(Milton!$A:$A, B29, Milton!$F:$F), 0)</f>
+        <v/>
+      </c>
+      <c r="V29" s="59" t="n"/>
       <c r="W29" s="9" t="n"/>
-      <c r="X29" s="22" t="n"/>
+      <c r="X29" s="21" t="n"/>
+      <c r="Y29" s="9" t="n"/>
+      <c r="Z29" s="21" t="n"/>
+      <c r="AA29" s="9" t="n"/>
+      <c r="AB29" s="22" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="55" t="n"/>
@@ -2630,12 +2934,22 @@
         <v/>
       </c>
       <c r="R30" s="23" t="n"/>
-      <c r="S30" s="9" t="n"/>
-      <c r="T30" s="23" t="n"/>
-      <c r="U30" s="9" t="n"/>
-      <c r="V30" s="23" t="n"/>
+      <c r="S30" s="59">
+        <f>IFERROR(SUMIF(Oshawa!$A:$A, B30, Oshawa!$F:$F), 0)</f>
+        <v/>
+      </c>
+      <c r="T30" s="59" t="n"/>
+      <c r="U30" s="59">
+        <f>IFERROR(SUMIF(Milton!$A:$A, B30, Milton!$F:$F), 0)</f>
+        <v/>
+      </c>
+      <c r="V30" s="59" t="n"/>
       <c r="W30" s="9" t="n"/>
       <c r="X30" s="23" t="n"/>
+      <c r="Y30" s="9" t="n"/>
+      <c r="Z30" s="23" t="n"/>
+      <c r="AA30" s="9" t="n"/>
+      <c r="AB30" s="23" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="55" t="n"/>
@@ -2684,12 +2998,22 @@
         <v/>
       </c>
       <c r="R31" s="23" t="n"/>
-      <c r="S31" s="9" t="n"/>
-      <c r="T31" s="23" t="n"/>
-      <c r="U31" s="9" t="n"/>
-      <c r="V31" s="23" t="n"/>
+      <c r="S31" s="59">
+        <f>IFERROR(SUMIF(Oshawa!$A:$A, B31, Oshawa!$F:$F), 0)</f>
+        <v/>
+      </c>
+      <c r="T31" s="59" t="n"/>
+      <c r="U31" s="59">
+        <f>IFERROR(SUMIF(Milton!$A:$A, B31, Milton!$F:$F), 0)</f>
+        <v/>
+      </c>
+      <c r="V31" s="59" t="n"/>
       <c r="W31" s="9" t="n"/>
       <c r="X31" s="23" t="n"/>
+      <c r="Y31" s="9" t="n"/>
+      <c r="Z31" s="23" t="n"/>
+      <c r="AA31" s="9" t="n"/>
+      <c r="AB31" s="23" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="55" t="n"/>
@@ -2738,12 +3062,22 @@
         <v/>
       </c>
       <c r="R32" s="23" t="n"/>
-      <c r="S32" s="9" t="n"/>
-      <c r="T32" s="23" t="n"/>
-      <c r="U32" s="9" t="n"/>
-      <c r="V32" s="23" t="n"/>
+      <c r="S32" s="59">
+        <f>IFERROR(SUMIF(Oshawa!$A:$A, B32, Oshawa!$F:$F), 0)</f>
+        <v/>
+      </c>
+      <c r="T32" s="59" t="n"/>
+      <c r="U32" s="59">
+        <f>IFERROR(SUMIF(Milton!$A:$A, B32, Milton!$F:$F), 0)</f>
+        <v/>
+      </c>
+      <c r="V32" s="59" t="n"/>
       <c r="W32" s="9" t="n"/>
       <c r="X32" s="23" t="n"/>
+      <c r="Y32" s="9" t="n"/>
+      <c r="Z32" s="23" t="n"/>
+      <c r="AA32" s="9" t="n"/>
+      <c r="AB32" s="23" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="55" t="n"/>
@@ -2792,12 +3126,22 @@
         <v/>
       </c>
       <c r="R33" s="23" t="n"/>
-      <c r="S33" s="9" t="n"/>
-      <c r="T33" s="23" t="n"/>
-      <c r="U33" s="9" t="n"/>
-      <c r="V33" s="23" t="n"/>
+      <c r="S33" s="59">
+        <f>IFERROR(SUMIF(Oshawa!$A:$A, B33, Oshawa!$F:$F), 0)</f>
+        <v/>
+      </c>
+      <c r="T33" s="59" t="n"/>
+      <c r="U33" s="59">
+        <f>IFERROR(SUMIF(Milton!$A:$A, B33, Milton!$F:$F), 0)</f>
+        <v/>
+      </c>
+      <c r="V33" s="59" t="n"/>
       <c r="W33" s="9" t="n"/>
       <c r="X33" s="23" t="n"/>
+      <c r="Y33" s="9" t="n"/>
+      <c r="Z33" s="23" t="n"/>
+      <c r="AA33" s="9" t="n"/>
+      <c r="AB33" s="23" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="55" t="n"/>
@@ -2846,12 +3190,22 @@
         <v/>
       </c>
       <c r="R34" s="23" t="n"/>
-      <c r="S34" s="9" t="n"/>
-      <c r="T34" s="23" t="n"/>
-      <c r="U34" s="9" t="n"/>
-      <c r="V34" s="23" t="n"/>
+      <c r="S34" s="59">
+        <f>IFERROR(SUMIF(Oshawa!$A:$A, B34, Oshawa!$F:$F), 0)</f>
+        <v/>
+      </c>
+      <c r="T34" s="59" t="n"/>
+      <c r="U34" s="59">
+        <f>IFERROR(SUMIF(Milton!$A:$A, B34, Milton!$F:$F), 0)</f>
+        <v/>
+      </c>
+      <c r="V34" s="59" t="n"/>
       <c r="W34" s="9" t="n"/>
       <c r="X34" s="23" t="n"/>
+      <c r="Y34" s="9" t="n"/>
+      <c r="Z34" s="23" t="n"/>
+      <c r="AA34" s="9" t="n"/>
+      <c r="AB34" s="23" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="55" t="n"/>
@@ -2900,12 +3254,22 @@
         <v/>
       </c>
       <c r="R35" s="23" t="n"/>
-      <c r="S35" s="9" t="n"/>
-      <c r="T35" s="23" t="n"/>
-      <c r="U35" s="9" t="n"/>
-      <c r="V35" s="23" t="n"/>
+      <c r="S35" s="59">
+        <f>IFERROR(SUMIF(Oshawa!$A:$A, B35, Oshawa!$F:$F), 0)</f>
+        <v/>
+      </c>
+      <c r="T35" s="59" t="n"/>
+      <c r="U35" s="59">
+        <f>IFERROR(SUMIF(Milton!$A:$A, B35, Milton!$F:$F), 0)</f>
+        <v/>
+      </c>
+      <c r="V35" s="59" t="n"/>
       <c r="W35" s="9" t="n"/>
       <c r="X35" s="23" t="n"/>
+      <c r="Y35" s="9" t="n"/>
+      <c r="Z35" s="23" t="n"/>
+      <c r="AA35" s="9" t="n"/>
+      <c r="AB35" s="23" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="55" t="n"/>
@@ -2954,12 +3318,22 @@
         <v/>
       </c>
       <c r="R36" s="24" t="n"/>
-      <c r="S36" s="9" t="n"/>
-      <c r="T36" s="24" t="n"/>
-      <c r="U36" s="9" t="n"/>
-      <c r="V36" s="24" t="n"/>
+      <c r="S36" s="59">
+        <f>IFERROR(SUMIF(Oshawa!$A:$A, B36, Oshawa!$F:$F), 0)</f>
+        <v/>
+      </c>
+      <c r="T36" s="59" t="n"/>
+      <c r="U36" s="59">
+        <f>IFERROR(SUMIF(Milton!$A:$A, B36, Milton!$F:$F), 0)</f>
+        <v/>
+      </c>
+      <c r="V36" s="59" t="n"/>
       <c r="W36" s="9" t="n"/>
       <c r="X36" s="24" t="n"/>
+      <c r="Y36" s="9" t="n"/>
+      <c r="Z36" s="24" t="n"/>
+      <c r="AA36" s="9" t="n"/>
+      <c r="AB36" s="24" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="55" t="n"/>
@@ -3008,12 +3382,22 @@
         <v/>
       </c>
       <c r="R37" s="24" t="n"/>
-      <c r="S37" s="9" t="n"/>
-      <c r="T37" s="24" t="n"/>
-      <c r="U37" s="9" t="n"/>
-      <c r="V37" s="24" t="n"/>
+      <c r="S37" s="58">
+        <f>IFERROR(SUMIF(Oshawa!$A:$A, B37, Oshawa!$F:$F), 0)</f>
+        <v/>
+      </c>
+      <c r="T37" s="58" t="n"/>
+      <c r="U37" s="58">
+        <f>IFERROR(SUMIF(Milton!$A:$A, B37, Milton!$F:$F), 0)</f>
+        <v/>
+      </c>
+      <c r="V37" s="58" t="n"/>
       <c r="W37" s="9" t="n"/>
       <c r="X37" s="24" t="n"/>
+      <c r="Y37" s="9" t="n"/>
+      <c r="Z37" s="24" t="n"/>
+      <c r="AA37" s="9" t="n"/>
+      <c r="AB37" s="24" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="55" t="n"/>
@@ -3062,12 +3446,22 @@
         <v/>
       </c>
       <c r="R38" s="24" t="n"/>
-      <c r="S38" s="9" t="n"/>
-      <c r="T38" s="24" t="n"/>
-      <c r="U38" s="9" t="n"/>
-      <c r="V38" s="24" t="n"/>
+      <c r="S38" s="58">
+        <f>IFERROR(SUMIF(Oshawa!$A:$A, B38, Oshawa!$F:$F), 0)</f>
+        <v/>
+      </c>
+      <c r="T38" s="58" t="n"/>
+      <c r="U38" s="58">
+        <f>IFERROR(SUMIF(Milton!$A:$A, B38, Milton!$F:$F), 0)</f>
+        <v/>
+      </c>
+      <c r="V38" s="58" t="n"/>
       <c r="W38" s="9" t="n"/>
       <c r="X38" s="24" t="n"/>
+      <c r="Y38" s="9" t="n"/>
+      <c r="Z38" s="24" t="n"/>
+      <c r="AA38" s="9" t="n"/>
+      <c r="AB38" s="24" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="55" t="n"/>
@@ -3116,12 +3510,22 @@
         <v/>
       </c>
       <c r="R39" s="24" t="n"/>
-      <c r="S39" s="9" t="n"/>
-      <c r="T39" s="24" t="n"/>
-      <c r="U39" s="9" t="n"/>
-      <c r="V39" s="24" t="n"/>
+      <c r="S39" s="58">
+        <f>IFERROR(SUMIF(Oshawa!$A:$A, B39, Oshawa!$F:$F), 0)</f>
+        <v/>
+      </c>
+      <c r="T39" s="58" t="n"/>
+      <c r="U39" s="58">
+        <f>IFERROR(SUMIF(Milton!$A:$A, B39, Milton!$F:$F), 0)</f>
+        <v/>
+      </c>
+      <c r="V39" s="58" t="n"/>
       <c r="W39" s="9" t="n"/>
       <c r="X39" s="24" t="n"/>
+      <c r="Y39" s="9" t="n"/>
+      <c r="Z39" s="24" t="n"/>
+      <c r="AA39" s="9" t="n"/>
+      <c r="AB39" s="24" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="55" t="n"/>
@@ -3170,12 +3574,22 @@
         <v/>
       </c>
       <c r="R40" s="24" t="n"/>
-      <c r="S40" s="9" t="n"/>
-      <c r="T40" s="24" t="n"/>
-      <c r="U40" s="9" t="n"/>
-      <c r="V40" s="24" t="n"/>
+      <c r="S40" s="58">
+        <f>IFERROR(SUMIF(Oshawa!$A:$A, B40, Oshawa!$F:$F), 0)</f>
+        <v/>
+      </c>
+      <c r="T40" s="58" t="n"/>
+      <c r="U40" s="58">
+        <f>IFERROR(SUMIF(Milton!$A:$A, B40, Milton!$F:$F), 0)</f>
+        <v/>
+      </c>
+      <c r="V40" s="58" t="n"/>
       <c r="W40" s="9" t="n"/>
       <c r="X40" s="24" t="n"/>
+      <c r="Y40" s="9" t="n"/>
+      <c r="Z40" s="24" t="n"/>
+      <c r="AA40" s="9" t="n"/>
+      <c r="AB40" s="24" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="55" t="n"/>
@@ -3224,12 +3638,22 @@
         <v/>
       </c>
       <c r="R41" s="24" t="n"/>
-      <c r="S41" s="24" t="n"/>
-      <c r="T41" s="24" t="n"/>
-      <c r="U41" s="24" t="n"/>
-      <c r="V41" s="24" t="n"/>
+      <c r="S41" s="59">
+        <f>IFERROR(SUMIF(Oshawa!$A:$A, B41, Oshawa!$F:$F), 0)</f>
+        <v/>
+      </c>
+      <c r="T41" s="59" t="n"/>
+      <c r="U41" s="59">
+        <f>IFERROR(SUMIF(Milton!$A:$A, B41, Milton!$F:$F), 0)</f>
+        <v/>
+      </c>
+      <c r="V41" s="59" t="n"/>
       <c r="W41" s="24" t="n"/>
       <c r="X41" s="24" t="n"/>
+      <c r="Y41" s="24" t="n"/>
+      <c r="Z41" s="24" t="n"/>
+      <c r="AA41" s="24" t="n"/>
+      <c r="AB41" s="24" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="55" t="n"/>
@@ -3278,12 +3702,22 @@
         <v/>
       </c>
       <c r="R42" s="24" t="n"/>
-      <c r="S42" s="24" t="n"/>
-      <c r="T42" s="24" t="n"/>
-      <c r="U42" s="24" t="n"/>
-      <c r="V42" s="24" t="n"/>
+      <c r="S42" s="59">
+        <f>IFERROR(SUMIF(Oshawa!$A:$A, B42, Oshawa!$F:$F), 0)</f>
+        <v/>
+      </c>
+      <c r="T42" s="59" t="n"/>
+      <c r="U42" s="59">
+        <f>IFERROR(SUMIF(Milton!$A:$A, B42, Milton!$F:$F), 0)</f>
+        <v/>
+      </c>
+      <c r="V42" s="59" t="n"/>
       <c r="W42" s="24" t="n"/>
       <c r="X42" s="24" t="n"/>
+      <c r="Y42" s="24" t="n"/>
+      <c r="Z42" s="24" t="n"/>
+      <c r="AA42" s="24" t="n"/>
+      <c r="AB42" s="24" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="55" t="n"/>
@@ -3332,12 +3766,22 @@
         <v/>
       </c>
       <c r="R43" s="24" t="n"/>
-      <c r="S43" s="24" t="n"/>
-      <c r="T43" s="24" t="n"/>
-      <c r="U43" s="24" t="n"/>
-      <c r="V43" s="24" t="n"/>
+      <c r="S43" s="59">
+        <f>IFERROR(SUMIF(Oshawa!$A:$A, B43, Oshawa!$F:$F), 0)</f>
+        <v/>
+      </c>
+      <c r="T43" s="59" t="n"/>
+      <c r="U43" s="59">
+        <f>IFERROR(SUMIF(Milton!$A:$A, B43, Milton!$F:$F), 0)</f>
+        <v/>
+      </c>
+      <c r="V43" s="59" t="n"/>
       <c r="W43" s="24" t="n"/>
       <c r="X43" s="24" t="n"/>
+      <c r="Y43" s="24" t="n"/>
+      <c r="Z43" s="24" t="n"/>
+      <c r="AA43" s="24" t="n"/>
+      <c r="AB43" s="24" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="55" t="n"/>
@@ -3386,12 +3830,22 @@
         <v/>
       </c>
       <c r="R44" s="24" t="n"/>
-      <c r="S44" s="24" t="n"/>
-      <c r="T44" s="24" t="n"/>
-      <c r="U44" s="24" t="n"/>
-      <c r="V44" s="24" t="n"/>
+      <c r="S44" s="59">
+        <f>IFERROR(SUMIF(Oshawa!$A:$A, B44, Oshawa!$F:$F), 0)</f>
+        <v/>
+      </c>
+      <c r="T44" s="59" t="n"/>
+      <c r="U44" s="59">
+        <f>IFERROR(SUMIF(Milton!$A:$A, B44, Milton!$F:$F), 0)</f>
+        <v/>
+      </c>
+      <c r="V44" s="59" t="n"/>
       <c r="W44" s="24" t="n"/>
       <c r="X44" s="24" t="n"/>
+      <c r="Y44" s="24" t="n"/>
+      <c r="Z44" s="24" t="n"/>
+      <c r="AA44" s="24" t="n"/>
+      <c r="AB44" s="24" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="56" t="n"/>
@@ -3440,12 +3894,22 @@
         <v/>
       </c>
       <c r="R45" s="24" t="n"/>
-      <c r="S45" s="24" t="n"/>
-      <c r="T45" s="24" t="n"/>
-      <c r="U45" s="24" t="n"/>
-      <c r="V45" s="24" t="n"/>
+      <c r="S45" s="59">
+        <f>IFERROR(SUMIF(Oshawa!$A:$A, B45, Oshawa!$F:$F), 0)</f>
+        <v/>
+      </c>
+      <c r="T45" s="59" t="n"/>
+      <c r="U45" s="59">
+        <f>IFERROR(SUMIF(Milton!$A:$A, B45, Milton!$F:$F), 0)</f>
+        <v/>
+      </c>
+      <c r="V45" s="59" t="n"/>
       <c r="W45" s="24" t="n"/>
       <c r="X45" s="24" t="n"/>
+      <c r="Y45" s="24" t="n"/>
+      <c r="Z45" s="24" t="n"/>
+      <c r="AA45" s="24" t="n"/>
+      <c r="AB45" s="24" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="48" t="inlineStr">
@@ -3498,20 +3962,30 @@
         <v/>
       </c>
       <c r="R46" s="10" t="n"/>
-      <c r="S46" s="11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="T46" s="9" t="n"/>
-      <c r="U46" s="9" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="V46" s="12" t="n"/>
-      <c r="W46" s="12" t="n"/>
-      <c r="X46" s="13" t="n"/>
+      <c r="S46" s="58">
+        <f>IFERROR(SUMIF(Oshawa!$A:$A, B46, Oshawa!$F:$F), 0)</f>
+        <v/>
+      </c>
+      <c r="T46" s="58" t="n"/>
+      <c r="U46" s="58">
+        <f>IFERROR(SUMIF(Milton!$A:$A, B46, Milton!$F:$F), 0)</f>
+        <v/>
+      </c>
+      <c r="V46" s="58" t="n"/>
+      <c r="W46" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="X46" s="9" t="n"/>
+      <c r="Y46" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Z46" s="12" t="n"/>
+      <c r="AA46" s="12" t="n"/>
+      <c r="AB46" s="13" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="49" t="n"/>
@@ -3560,20 +4034,30 @@
         <v/>
       </c>
       <c r="R47" s="10" t="n"/>
-      <c r="S47" s="11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="T47" s="9" t="n"/>
-      <c r="U47" s="9" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="V47" s="12" t="n"/>
-      <c r="W47" s="12" t="n"/>
-      <c r="X47" s="13" t="n"/>
+      <c r="S47" s="58">
+        <f>IFERROR(SUMIF(Oshawa!$A:$A, B47, Oshawa!$F:$F), 0)</f>
+        <v/>
+      </c>
+      <c r="T47" s="58" t="n"/>
+      <c r="U47" s="58">
+        <f>IFERROR(SUMIF(Milton!$A:$A, B47, Milton!$F:$F), 0)</f>
+        <v/>
+      </c>
+      <c r="V47" s="58" t="n"/>
+      <c r="W47" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="X47" s="9" t="n"/>
+      <c r="Y47" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Z47" s="12" t="n"/>
+      <c r="AA47" s="12" t="n"/>
+      <c r="AB47" s="13" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="49" t="n"/>
@@ -3622,20 +4106,30 @@
         <v/>
       </c>
       <c r="R48" s="10" t="n"/>
-      <c r="S48" s="11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="T48" s="9" t="n"/>
-      <c r="U48" s="9" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="V48" s="12" t="n"/>
-      <c r="W48" s="12" t="n"/>
-      <c r="X48" s="13" t="n"/>
+      <c r="S48" s="58">
+        <f>IFERROR(SUMIF(Oshawa!$A:$A, B48, Oshawa!$F:$F), 0)</f>
+        <v/>
+      </c>
+      <c r="T48" s="58" t="n"/>
+      <c r="U48" s="58">
+        <f>IFERROR(SUMIF(Milton!$A:$A, B48, Milton!$F:$F), 0)</f>
+        <v/>
+      </c>
+      <c r="V48" s="58" t="n"/>
+      <c r="W48" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="X48" s="9" t="n"/>
+      <c r="Y48" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Z48" s="12" t="n"/>
+      <c r="AA48" s="12" t="n"/>
+      <c r="AB48" s="13" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="49" t="n"/>
@@ -3684,20 +4178,30 @@
         <v/>
       </c>
       <c r="R49" s="10" t="n"/>
-      <c r="S49" s="11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="T49" s="9" t="n"/>
-      <c r="U49" s="9" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="V49" s="12" t="n"/>
-      <c r="W49" s="12" t="n"/>
-      <c r="X49" s="13" t="n"/>
+      <c r="S49" s="58">
+        <f>IFERROR(SUMIF(Oshawa!$A:$A, B49, Oshawa!$F:$F), 0)</f>
+        <v/>
+      </c>
+      <c r="T49" s="58" t="n"/>
+      <c r="U49" s="58">
+        <f>IFERROR(SUMIF(Milton!$A:$A, B49, Milton!$F:$F), 0)</f>
+        <v/>
+      </c>
+      <c r="V49" s="58" t="n"/>
+      <c r="W49" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="X49" s="9" t="n"/>
+      <c r="Y49" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Z49" s="12" t="n"/>
+      <c r="AA49" s="12" t="n"/>
+      <c r="AB49" s="13" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="49" t="n"/>
@@ -3746,20 +4250,30 @@
         <v/>
       </c>
       <c r="R50" s="10" t="n"/>
-      <c r="S50" s="11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="T50" s="9" t="n"/>
-      <c r="U50" s="9" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="V50" s="12" t="n"/>
-      <c r="W50" s="12" t="n"/>
-      <c r="X50" s="13" t="n"/>
+      <c r="S50" s="58">
+        <f>IFERROR(SUMIF(Oshawa!$A:$A, B50, Oshawa!$F:$F), 0)</f>
+        <v/>
+      </c>
+      <c r="T50" s="58" t="n"/>
+      <c r="U50" s="58">
+        <f>IFERROR(SUMIF(Milton!$A:$A, B50, Milton!$F:$F), 0)</f>
+        <v/>
+      </c>
+      <c r="V50" s="58" t="n"/>
+      <c r="W50" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="X50" s="9" t="n"/>
+      <c r="Y50" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Z50" s="12" t="n"/>
+      <c r="AA50" s="12" t="n"/>
+      <c r="AB50" s="13" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="49" t="n"/>
@@ -3808,20 +4322,30 @@
         <v/>
       </c>
       <c r="R51" s="10" t="n"/>
-      <c r="S51" s="11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="T51" s="9" t="n"/>
-      <c r="U51" s="9" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="V51" s="12" t="n"/>
-      <c r="W51" s="12" t="n"/>
-      <c r="X51" s="13" t="n"/>
+      <c r="S51" s="58">
+        <f>IFERROR(SUMIF(Oshawa!$A:$A, B51, Oshawa!$F:$F), 0)</f>
+        <v/>
+      </c>
+      <c r="T51" s="58" t="n"/>
+      <c r="U51" s="58">
+        <f>IFERROR(SUMIF(Milton!$A:$A, B51, Milton!$F:$F), 0)</f>
+        <v/>
+      </c>
+      <c r="V51" s="58" t="n"/>
+      <c r="W51" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="X51" s="9" t="n"/>
+      <c r="Y51" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Z51" s="12" t="n"/>
+      <c r="AA51" s="12" t="n"/>
+      <c r="AB51" s="13" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="49" t="n"/>
@@ -3870,20 +4394,30 @@
         <v/>
       </c>
       <c r="R52" s="10" t="n"/>
-      <c r="S52" s="15" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="T52" s="16" t="n"/>
-      <c r="U52" s="16" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="V52" s="12" t="n"/>
-      <c r="W52" s="12" t="n"/>
-      <c r="X52" s="13" t="n"/>
+      <c r="S52" s="58">
+        <f>IFERROR(SUMIF(Oshawa!$A:$A, B52, Oshawa!$F:$F), 0)</f>
+        <v/>
+      </c>
+      <c r="T52" s="58" t="n"/>
+      <c r="U52" s="58">
+        <f>IFERROR(SUMIF(Milton!$A:$A, B52, Milton!$F:$F), 0)</f>
+        <v/>
+      </c>
+      <c r="V52" s="58" t="n"/>
+      <c r="W52" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="X52" s="16" t="n"/>
+      <c r="Y52" s="16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Z52" s="12" t="n"/>
+      <c r="AA52" s="12" t="n"/>
+      <c r="AB52" s="13" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="49" t="n"/>
@@ -3932,20 +4466,30 @@
         <v/>
       </c>
       <c r="R53" s="10" t="n"/>
-      <c r="S53" s="11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="T53" s="9" t="n"/>
-      <c r="U53" s="9" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="V53" s="12" t="n"/>
-      <c r="W53" s="12" t="n"/>
-      <c r="X53" s="13" t="n"/>
+      <c r="S53" s="58">
+        <f>IFERROR(SUMIF(Oshawa!$A:$A, B53, Oshawa!$F:$F), 0)</f>
+        <v/>
+      </c>
+      <c r="T53" s="58" t="n"/>
+      <c r="U53" s="58">
+        <f>IFERROR(SUMIF(Milton!$A:$A, B53, Milton!$F:$F), 0)</f>
+        <v/>
+      </c>
+      <c r="V53" s="58" t="n"/>
+      <c r="W53" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="X53" s="9" t="n"/>
+      <c r="Y53" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Z53" s="12" t="n"/>
+      <c r="AA53" s="12" t="n"/>
+      <c r="AB53" s="13" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="49" t="n"/>
@@ -3994,20 +4538,30 @@
         <v/>
       </c>
       <c r="R54" s="10" t="n"/>
-      <c r="S54" s="11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="T54" s="9" t="n"/>
-      <c r="U54" s="9" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="V54" s="12" t="n"/>
-      <c r="W54" s="12" t="n"/>
-      <c r="X54" s="13" t="n"/>
+      <c r="S54" s="58">
+        <f>IFERROR(SUMIF(Oshawa!$A:$A, B54, Oshawa!$F:$F), 0)</f>
+        <v/>
+      </c>
+      <c r="T54" s="58" t="n"/>
+      <c r="U54" s="58">
+        <f>IFERROR(SUMIF(Milton!$A:$A, B54, Milton!$F:$F), 0)</f>
+        <v/>
+      </c>
+      <c r="V54" s="58" t="n"/>
+      <c r="W54" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="X54" s="9" t="n"/>
+      <c r="Y54" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Z54" s="12" t="n"/>
+      <c r="AA54" s="12" t="n"/>
+      <c r="AB54" s="13" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="49" t="n"/>
@@ -4056,20 +4610,30 @@
         <v/>
       </c>
       <c r="R55" s="10" t="n"/>
-      <c r="S55" s="11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="T55" s="9" t="n"/>
-      <c r="U55" s="9" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="V55" s="12" t="n"/>
-      <c r="W55" s="12" t="n"/>
-      <c r="X55" s="13" t="n"/>
+      <c r="S55" s="58">
+        <f>IFERROR(SUMIF(Oshawa!$A:$A, B55, Oshawa!$F:$F), 0)</f>
+        <v/>
+      </c>
+      <c r="T55" s="58" t="n"/>
+      <c r="U55" s="58">
+        <f>IFERROR(SUMIF(Milton!$A:$A, B55, Milton!$F:$F), 0)</f>
+        <v/>
+      </c>
+      <c r="V55" s="58" t="n"/>
+      <c r="W55" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="X55" s="9" t="n"/>
+      <c r="Y55" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Z55" s="12" t="n"/>
+      <c r="AA55" s="12" t="n"/>
+      <c r="AB55" s="13" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="49" t="n"/>
@@ -4118,20 +4682,30 @@
         <v/>
       </c>
       <c r="R56" s="10" t="n"/>
-      <c r="S56" s="11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="T56" s="9" t="n"/>
-      <c r="U56" s="9" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="V56" s="12" t="n"/>
-      <c r="W56" s="12" t="n"/>
-      <c r="X56" s="13" t="n"/>
+      <c r="S56" s="58">
+        <f>IFERROR(SUMIF(Oshawa!$A:$A, B56, Oshawa!$F:$F), 0)</f>
+        <v/>
+      </c>
+      <c r="T56" s="58" t="n"/>
+      <c r="U56" s="58">
+        <f>IFERROR(SUMIF(Milton!$A:$A, B56, Milton!$F:$F), 0)</f>
+        <v/>
+      </c>
+      <c r="V56" s="58" t="n"/>
+      <c r="W56" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="X56" s="9" t="n"/>
+      <c r="Y56" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Z56" s="12" t="n"/>
+      <c r="AA56" s="12" t="n"/>
+      <c r="AB56" s="13" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="49" t="n"/>
@@ -4180,20 +4754,30 @@
         <v/>
       </c>
       <c r="R57" s="29" t="n"/>
-      <c r="S57" s="37" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="T57" s="26" t="n"/>
-      <c r="U57" s="26" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="V57" s="27" t="n"/>
-      <c r="W57" s="27" t="n"/>
-      <c r="X57" s="13" t="n"/>
+      <c r="S57" s="60">
+        <f>IFERROR(SUMIF(Oshawa!$A:$A, B57, Oshawa!$F:$F), 0)</f>
+        <v/>
+      </c>
+      <c r="T57" s="60" t="n"/>
+      <c r="U57" s="60">
+        <f>IFERROR(SUMIF(Milton!$A:$A, B57, Milton!$F:$F), 0)</f>
+        <v/>
+      </c>
+      <c r="V57" s="60" t="n"/>
+      <c r="W57" s="37" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="X57" s="26" t="n"/>
+      <c r="Y57" s="26" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Z57" s="27" t="n"/>
+      <c r="AA57" s="27" t="n"/>
+      <c r="AB57" s="13" t="n"/>
     </row>
     <row r="58" ht="15" customHeight="1" thickBot="1">
       <c r="A58" s="49" t="n"/>
@@ -4242,12 +4826,22 @@
         <v/>
       </c>
       <c r="R58" s="34" t="n"/>
-      <c r="S58" s="17" t="n"/>
-      <c r="T58" s="18" t="n"/>
-      <c r="U58" s="17" t="n"/>
-      <c r="V58" s="19" t="n"/>
-      <c r="W58" s="35" t="n"/>
-      <c r="X58" s="20" t="n"/>
+      <c r="S58" s="61">
+        <f>SUM(S46:S57)</f>
+        <v/>
+      </c>
+      <c r="T58" s="61" t="n"/>
+      <c r="U58" s="61">
+        <f>SUM(U46:U57)</f>
+        <v/>
+      </c>
+      <c r="V58" s="61" t="n"/>
+      <c r="W58" s="17" t="n"/>
+      <c r="X58" s="18" t="n"/>
+      <c r="Y58" s="17" t="n"/>
+      <c r="Z58" s="19" t="n"/>
+      <c r="AA58" s="35" t="n"/>
+      <c r="AB58" s="20" t="n"/>
     </row>
     <row r="59" ht="15" customHeight="1">
       <c r="A59" s="51" t="inlineStr">
@@ -4308,18 +4902,30 @@
         </is>
       </c>
       <c r="R59" s="38" t="n"/>
-      <c r="S59" s="9">
+      <c r="S59" s="58" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="T59" s="58" t="n"/>
+      <c r="U59" s="58" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="V59" s="58" t="n"/>
+      <c r="W59" s="9">
         <f>IFERROR(SUMIF('Karachi Food Court'!$A:$A, B59, 'Karachi Food Court'!$F:$F), 0)</f>
         <v/>
       </c>
-      <c r="T59" s="38" t="n"/>
-      <c r="U59" s="9">
+      <c r="X59" s="38" t="n"/>
+      <c r="Y59" s="9">
         <f>IFERROR(SUMIF('Karachi Kabab Wala'!$A:$A, B59, 'Karachi Kabab Wala'!$F:$F), 0)</f>
         <v/>
       </c>
-      <c r="V59" s="28" t="n"/>
-      <c r="W59" s="28" t="n"/>
-      <c r="X59" s="28" t="n"/>
+      <c r="Z59" s="28" t="n"/>
+      <c r="AA59" s="28" t="n"/>
+      <c r="AB59" s="28" t="n"/>
     </row>
     <row r="60" ht="15" customHeight="1">
       <c r="A60" s="55" t="n"/>
@@ -4376,18 +4982,30 @@
         </is>
       </c>
       <c r="R60" s="24" t="n"/>
-      <c r="S60" s="9">
+      <c r="S60" s="58" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="T60" s="58" t="n"/>
+      <c r="U60" s="58" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="V60" s="58" t="n"/>
+      <c r="W60" s="9">
         <f>IFERROR(SUMIF('Karachi Food Court'!$A:$A, B60, 'Karachi Food Court'!$F:$F), 0)</f>
         <v/>
       </c>
-      <c r="T60" s="24" t="n"/>
-      <c r="U60" s="9">
+      <c r="X60" s="24" t="n"/>
+      <c r="Y60" s="9">
         <f>IFERROR(SUMIF('Karachi Kabab Wala'!$A:$A, B60, 'Karachi Kabab Wala'!$F:$F), 0)</f>
         <v/>
       </c>
-      <c r="V60" s="28" t="n"/>
-      <c r="W60" s="28" t="n"/>
-      <c r="X60" s="28" t="n"/>
+      <c r="Z60" s="28" t="n"/>
+      <c r="AA60" s="28" t="n"/>
+      <c r="AB60" s="28" t="n"/>
     </row>
     <row r="61" ht="14.45" customHeight="1">
       <c r="A61" s="55" t="n"/>
@@ -4444,21 +5062,33 @@
         </is>
       </c>
       <c r="R61" s="9" t="n"/>
-      <c r="S61" s="9">
+      <c r="S61" s="58" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="T61" s="58" t="n"/>
+      <c r="U61" s="58" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="V61" s="58" t="n"/>
+      <c r="W61" s="9">
         <f>IFERROR(SUMIF('Karachi Food Court'!$A:$A, B61, 'Karachi Food Court'!$F:$F), 0)</f>
         <v/>
       </c>
-      <c r="T61" s="10" t="n"/>
-      <c r="U61" s="9">
+      <c r="X61" s="10" t="n"/>
+      <c r="Y61" s="9">
         <f>IFERROR(SUMIF('Karachi Kabab Wala'!$A:$A, B61, 'Karachi Kabab Wala'!$F:$F), 0)</f>
         <v/>
       </c>
-      <c r="V61" s="10" t="n"/>
-      <c r="W61" s="9">
+      <c r="Z61" s="10" t="n"/>
+      <c r="AA61" s="9">
         <f>IFERROR(SUMIF('Karachi Kabab Wala - Queen'!$A:$A, B61, 'Karachi Kabab Wala - Queen'!$F:$F), 0)</f>
         <v/>
       </c>
-      <c r="X61" s="10" t="n"/>
+      <c r="AB61" s="10" t="n"/>
     </row>
     <row r="62">
       <c r="A62" s="55" t="n"/>
@@ -4515,21 +5145,33 @@
         </is>
       </c>
       <c r="R62" s="9" t="n"/>
-      <c r="S62" s="9">
+      <c r="S62" s="58" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="T62" s="58" t="n"/>
+      <c r="U62" s="58" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="V62" s="58" t="n"/>
+      <c r="W62" s="9">
         <f>IFERROR(SUMIF('Karachi Food Court'!$A:$A, B62, 'Karachi Food Court'!$F:$F), 0)</f>
         <v/>
       </c>
-      <c r="T62" s="10" t="n"/>
-      <c r="U62" s="9">
+      <c r="X62" s="10" t="n"/>
+      <c r="Y62" s="9">
         <f>IFERROR(SUMIF('Karachi Kabab Wala'!$A:$A, B62, 'Karachi Kabab Wala'!$F:$F), 0)</f>
         <v/>
       </c>
-      <c r="V62" s="10" t="n"/>
-      <c r="W62" s="9">
+      <c r="Z62" s="10" t="n"/>
+      <c r="AA62" s="9">
         <f>IFERROR(SUMIF('Karachi Kabab Wala - Queen'!$A:$A, B62, 'Karachi Kabab Wala - Queen'!$F:$F), 0)</f>
         <v/>
       </c>
-      <c r="X62" s="10" t="n"/>
+      <c r="AB62" s="10" t="n"/>
     </row>
     <row r="63">
       <c r="A63" s="55" t="n"/>
@@ -4586,21 +5228,33 @@
         </is>
       </c>
       <c r="R63" s="9" t="n"/>
-      <c r="S63" s="9">
+      <c r="S63" s="58" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="T63" s="58" t="n"/>
+      <c r="U63" s="58" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="V63" s="58" t="n"/>
+      <c r="W63" s="9">
         <f>IFERROR(SUMIF('Karachi Food Court'!$A:$A, B63, 'Karachi Food Court'!$F:$F), 0)</f>
         <v/>
       </c>
-      <c r="T63" s="10" t="n"/>
-      <c r="U63" s="9">
+      <c r="X63" s="10" t="n"/>
+      <c r="Y63" s="9">
         <f>IFERROR(SUMIF('Karachi Kabab Wala'!$A:$A, B63, 'Karachi Kabab Wala'!$F:$F), 0)</f>
         <v/>
       </c>
-      <c r="V63" s="10" t="n"/>
-      <c r="W63" s="9">
+      <c r="Z63" s="10" t="n"/>
+      <c r="AA63" s="9">
         <f>IFERROR(SUMIF('Karachi Kabab Wala - Queen'!$A:$A, B63, 'Karachi Kabab Wala - Queen'!$F:$F), 0)</f>
         <v/>
       </c>
-      <c r="X63" s="10" t="n"/>
+      <c r="AB63" s="10" t="n"/>
     </row>
     <row r="64">
       <c r="A64" s="55" t="n"/>
@@ -4657,21 +5311,33 @@
         </is>
       </c>
       <c r="R64" s="9" t="n"/>
-      <c r="S64" s="9">
+      <c r="S64" s="58" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="T64" s="58" t="n"/>
+      <c r="U64" s="58" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="V64" s="58" t="n"/>
+      <c r="W64" s="9">
         <f>IFERROR(SUMIF('Karachi Food Court'!$A:$A, B64, 'Karachi Food Court'!$F:$F), 0)</f>
         <v/>
       </c>
-      <c r="T64" s="10" t="n"/>
-      <c r="U64" s="9">
+      <c r="X64" s="10" t="n"/>
+      <c r="Y64" s="9">
         <f>IFERROR(SUMIF('Karachi Kabab Wala'!$A:$A, B64, 'Karachi Kabab Wala'!$F:$F), 0)</f>
         <v/>
       </c>
-      <c r="V64" s="10" t="n"/>
-      <c r="W64" s="9">
+      <c r="Z64" s="10" t="n"/>
+      <c r="AA64" s="9">
         <f>IFERROR(SUMIF('Karachi Kabab Wala - Queen'!$A:$A, B64, 'Karachi Kabab Wala - Queen'!$F:$F), 0)</f>
         <v/>
       </c>
-      <c r="X64" s="10" t="n"/>
+      <c r="AB64" s="10" t="n"/>
     </row>
     <row r="65">
       <c r="A65" s="55" t="n"/>
@@ -4728,21 +5394,33 @@
         </is>
       </c>
       <c r="R65" s="9" t="n"/>
-      <c r="S65" s="9">
+      <c r="S65" s="58" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="T65" s="58" t="n"/>
+      <c r="U65" s="58" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="V65" s="58" t="n"/>
+      <c r="W65" s="9">
         <f>IFERROR(SUMIF('Karachi Food Court'!$A:$A, B65, 'Karachi Food Court'!$F:$F), 0)</f>
         <v/>
       </c>
-      <c r="T65" s="10" t="n"/>
-      <c r="U65" s="9">
+      <c r="X65" s="10" t="n"/>
+      <c r="Y65" s="9">
         <f>IFERROR(SUMIF('Karachi Kabab Wala'!$A:$A, B65, 'Karachi Kabab Wala'!$F:$F), 0)</f>
         <v/>
       </c>
-      <c r="V65" s="10" t="n"/>
-      <c r="W65" s="9">
+      <c r="Z65" s="10" t="n"/>
+      <c r="AA65" s="9">
         <f>IFERROR(SUMIF('Karachi Kabab Wala - Queen'!$A:$A, B65, 'Karachi Kabab Wala - Queen'!$F:$F), 0)</f>
         <v/>
       </c>
-      <c r="X65" s="10" t="n"/>
+      <c r="AB65" s="10" t="n"/>
     </row>
     <row r="66">
       <c r="A66" s="55" t="n"/>
@@ -4799,21 +5477,33 @@
         </is>
       </c>
       <c r="R66" s="9" t="n"/>
-      <c r="S66" s="9">
+      <c r="S66" s="58" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="T66" s="58" t="n"/>
+      <c r="U66" s="58" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="V66" s="58" t="n"/>
+      <c r="W66" s="9">
         <f>IFERROR(SUMIF('Karachi Food Court'!$A:$A, B66, 'Karachi Food Court'!$F:$F), 0)</f>
         <v/>
       </c>
-      <c r="T66" s="10" t="n"/>
-      <c r="U66" s="9">
+      <c r="X66" s="10" t="n"/>
+      <c r="Y66" s="9">
         <f>IFERROR(SUMIF('Karachi Kabab Wala'!$A:$A, B66, 'Karachi Kabab Wala'!$F:$F), 0)</f>
         <v/>
       </c>
-      <c r="V66" s="10" t="n"/>
-      <c r="W66" s="9">
+      <c r="Z66" s="10" t="n"/>
+      <c r="AA66" s="9">
         <f>IFERROR(SUMIF('Karachi Kabab Wala - Queen'!$A:$A, B66, 'Karachi Kabab Wala - Queen'!$F:$F), 0)</f>
         <v/>
       </c>
-      <c r="X66" s="10" t="n"/>
+      <c r="AB66" s="10" t="n"/>
     </row>
     <row r="67">
       <c r="A67" s="55" t="n"/>
@@ -4870,21 +5560,33 @@
         </is>
       </c>
       <c r="R67" s="9" t="n"/>
-      <c r="S67" s="9">
+      <c r="S67" s="58" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="T67" s="58" t="n"/>
+      <c r="U67" s="58" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="V67" s="58" t="n"/>
+      <c r="W67" s="9">
         <f>IFERROR(SUMIF('Karachi Food Court'!$A:$A, B67, 'Karachi Food Court'!$F:$F), 0)</f>
         <v/>
       </c>
-      <c r="T67" s="10" t="n"/>
-      <c r="U67" s="9">
+      <c r="X67" s="10" t="n"/>
+      <c r="Y67" s="9">
         <f>IFERROR(SUMIF('Karachi Kabab Wala'!$A:$A, B67, 'Karachi Kabab Wala'!$F:$F), 0)</f>
         <v/>
       </c>
-      <c r="V67" s="10" t="n"/>
-      <c r="W67" s="9">
+      <c r="Z67" s="10" t="n"/>
+      <c r="AA67" s="9">
         <f>IFERROR(SUMIF('Karachi Kabab Wala - Queen'!$A:$A, B67, 'Karachi Kabab Wala - Queen'!$F:$F), 0)</f>
         <v/>
       </c>
-      <c r="X67" s="10" t="n"/>
+      <c r="AB67" s="10" t="n"/>
     </row>
     <row r="68">
       <c r="A68" s="55" t="n"/>
@@ -4941,21 +5643,33 @@
         </is>
       </c>
       <c r="R68" s="9" t="n"/>
-      <c r="S68" s="9">
+      <c r="S68" s="58" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="T68" s="58" t="n"/>
+      <c r="U68" s="58" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="V68" s="58" t="n"/>
+      <c r="W68" s="9">
         <f>IFERROR(SUMIF('Karachi Food Court'!$A:$A, B68, 'Karachi Food Court'!$F:$F), 0)</f>
         <v/>
       </c>
-      <c r="T68" s="10" t="n"/>
-      <c r="U68" s="9">
+      <c r="X68" s="10" t="n"/>
+      <c r="Y68" s="9">
         <f>IFERROR(SUMIF('Karachi Kabab Wala'!$A:$A, B68, 'Karachi Kabab Wala'!$F:$F), 0)</f>
         <v/>
       </c>
-      <c r="V68" s="10" t="n"/>
-      <c r="W68" s="9">
+      <c r="Z68" s="10" t="n"/>
+      <c r="AA68" s="9">
         <f>IFERROR(SUMIF('Karachi Kabab Wala - Queen'!$A:$A, B68, 'Karachi Kabab Wala - Queen'!$F:$F), 0)</f>
         <v/>
       </c>
-      <c r="X68" s="10" t="n"/>
+      <c r="AB68" s="10" t="n"/>
     </row>
     <row r="69">
       <c r="A69" s="55" t="n"/>
@@ -5012,21 +5726,33 @@
         </is>
       </c>
       <c r="R69" s="9" t="n"/>
-      <c r="S69" s="9">
+      <c r="S69" s="58" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="T69" s="58" t="n"/>
+      <c r="U69" s="58" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="V69" s="58" t="n"/>
+      <c r="W69" s="9">
         <f>IFERROR(SUMIF('Karachi Food Court'!$A:$A, B69, 'Karachi Food Court'!$F:$F), 0)</f>
         <v/>
       </c>
-      <c r="T69" s="10" t="n"/>
-      <c r="U69" s="9">
+      <c r="X69" s="10" t="n"/>
+      <c r="Y69" s="9">
         <f>IFERROR(SUMIF('Karachi Kabab Wala'!$A:$A, B69, 'Karachi Kabab Wala'!$F:$F), 0)</f>
         <v/>
       </c>
-      <c r="V69" s="10" t="n"/>
-      <c r="W69" s="9">
+      <c r="Z69" s="10" t="n"/>
+      <c r="AA69" s="9">
         <f>IFERROR(SUMIF('Karachi Kabab Wala - Queen'!$A:$A, B69, 'Karachi Kabab Wala - Queen'!$F:$F), 0)</f>
         <v/>
       </c>
-      <c r="X69" s="10" t="n"/>
+      <c r="AB69" s="10" t="n"/>
     </row>
     <row r="70">
       <c r="A70" s="55" t="n"/>
@@ -5083,21 +5809,33 @@
         </is>
       </c>
       <c r="R70" s="9" t="n"/>
-      <c r="S70" s="9">
+      <c r="S70" s="58" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="T70" s="58" t="n"/>
+      <c r="U70" s="58" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="V70" s="58" t="n"/>
+      <c r="W70" s="9">
         <f>IFERROR(SUMIF('Karachi Food Court'!$A:$A, B70, 'Karachi Food Court'!$F:$F), 0)</f>
         <v/>
       </c>
-      <c r="T70" s="10" t="n"/>
-      <c r="U70" s="9">
+      <c r="X70" s="10" t="n"/>
+      <c r="Y70" s="9">
         <f>IFERROR(SUMIF('Karachi Kabab Wala'!$A:$A, B70, 'Karachi Kabab Wala'!$F:$F), 0)</f>
         <v/>
       </c>
-      <c r="V70" s="10" t="n"/>
-      <c r="W70" s="9">
+      <c r="Z70" s="10" t="n"/>
+      <c r="AA70" s="9">
         <f>IFERROR(SUMIF('Karachi Kabab Wala - Queen'!$A:$A, B70, 'Karachi Kabab Wala - Queen'!$F:$F), 0)</f>
         <v/>
       </c>
-      <c r="X70" s="10" t="n"/>
+      <c r="AB70" s="10" t="n"/>
     </row>
     <row r="71">
       <c r="A71" s="55" t="n"/>
@@ -5154,21 +5892,33 @@
         </is>
       </c>
       <c r="R71" s="9" t="n"/>
-      <c r="S71" s="9">
+      <c r="S71" s="58" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="T71" s="58" t="n"/>
+      <c r="U71" s="58" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="V71" s="58" t="n"/>
+      <c r="W71" s="9">
         <f>IFERROR(SUMIF('Karachi Food Court'!$A:$A, B71, 'Karachi Food Court'!$F:$F), 0)</f>
         <v/>
       </c>
-      <c r="T71" s="10" t="n"/>
-      <c r="U71" s="9">
+      <c r="X71" s="10" t="n"/>
+      <c r="Y71" s="9">
         <f>IFERROR(SUMIF('Karachi Kabab Wala'!$A:$A, B71, 'Karachi Kabab Wala'!$F:$F), 0)</f>
         <v/>
       </c>
-      <c r="V71" s="10" t="n"/>
-      <c r="W71" s="9">
+      <c r="Z71" s="10" t="n"/>
+      <c r="AA71" s="9">
         <f>IFERROR(SUMIF('Karachi Kabab Wala - Queen'!$A:$A, B71, 'Karachi Kabab Wala - Queen'!$F:$F), 0)</f>
         <v/>
       </c>
-      <c r="X71" s="10" t="n"/>
+      <c r="AB71" s="10" t="n"/>
     </row>
     <row r="72">
       <c r="A72" s="55" t="n"/>
@@ -5225,21 +5975,33 @@
         </is>
       </c>
       <c r="R72" s="9" t="n"/>
-      <c r="S72" s="9">
+      <c r="S72" s="58" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="T72" s="58" t="n"/>
+      <c r="U72" s="58" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="V72" s="58" t="n"/>
+      <c r="W72" s="9">
         <f>IFERROR(SUMIF('Karachi Food Court'!$A:$A, B72, 'Karachi Food Court'!$F:$F), 0)</f>
         <v/>
       </c>
-      <c r="T72" s="10" t="n"/>
-      <c r="U72" s="9">
+      <c r="X72" s="10" t="n"/>
+      <c r="Y72" s="9">
         <f>IFERROR(SUMIF('Karachi Kabab Wala'!$A:$A, B72, 'Karachi Kabab Wala'!$F:$F), 0)</f>
         <v/>
       </c>
-      <c r="V72" s="10" t="n"/>
-      <c r="W72" s="9">
+      <c r="Z72" s="10" t="n"/>
+      <c r="AA72" s="9">
         <f>IFERROR(SUMIF('Karachi Kabab Wala - Queen'!$A:$A, B72, 'Karachi Kabab Wala - Queen'!$F:$F), 0)</f>
         <v/>
       </c>
-      <c r="X72" s="10" t="n"/>
+      <c r="AB72" s="10" t="n"/>
     </row>
     <row r="73">
       <c r="A73" s="55" t="n"/>
@@ -5272,22 +6034,22 @@
         </is>
       </c>
       <c r="R73" s="9" t="n"/>
-      <c r="S73" s="9" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="T73" s="9" t="n"/>
-      <c r="U73" s="9">
+      <c r="W73" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="X73" s="9" t="n"/>
+      <c r="Y73" s="9">
         <f>IFERROR(SUMIF('Karachi Kabab Wala'!$A:$A, B73, 'Karachi Kabab Wala'!$F:$F), 0)</f>
         <v/>
       </c>
-      <c r="V73" s="10" t="n"/>
-      <c r="W73" s="9">
+      <c r="Z73" s="10" t="n"/>
+      <c r="AA73" s="9">
         <f>IFERROR(SUMIF('Karachi Kabab Wala - Queen'!$A:$A, B73, 'Karachi Kabab Wala - Queen'!$F:$F), 0)</f>
         <v/>
       </c>
-      <c r="X73" s="10" t="n"/>
+      <c r="AB73" s="10" t="n"/>
     </row>
     <row r="74">
       <c r="A74" s="55" t="n"/>
@@ -5320,22 +6082,22 @@
         </is>
       </c>
       <c r="R74" s="9" t="n"/>
-      <c r="S74" s="9" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="T74" s="9" t="n"/>
-      <c r="U74" s="9">
+      <c r="W74" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="X74" s="9" t="n"/>
+      <c r="Y74" s="9">
         <f>IFERROR(SUMIF('Karachi Kabab Wala'!$A:$A, B74, 'Karachi Kabab Wala'!$F:$F), 0)</f>
         <v/>
       </c>
-      <c r="V74" s="10" t="n"/>
-      <c r="W74" s="9">
+      <c r="Z74" s="10" t="n"/>
+      <c r="AA74" s="9">
         <f>IFERROR(SUMIF('Karachi Kabab Wala - Queen'!$A:$A, B74, 'Karachi Kabab Wala - Queen'!$F:$F), 0)</f>
         <v/>
       </c>
-      <c r="X74" s="10" t="n"/>
+      <c r="AB74" s="10" t="n"/>
     </row>
     <row r="75">
       <c r="A75" s="55" t="n"/>
@@ -5368,22 +6130,22 @@
         </is>
       </c>
       <c r="R75" s="9" t="n"/>
-      <c r="S75" s="9" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="T75" s="9" t="n"/>
-      <c r="U75" s="9">
+      <c r="W75" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="X75" s="9" t="n"/>
+      <c r="Y75" s="9">
         <f>IFERROR(SUMIF('Karachi Kabab Wala'!$A:$A, B75, 'Karachi Kabab Wala'!$F:$F), 0)</f>
         <v/>
       </c>
-      <c r="V75" s="10" t="n"/>
-      <c r="W75" s="9">
+      <c r="Z75" s="10" t="n"/>
+      <c r="AA75" s="9">
         <f>IFERROR(SUMIF('Karachi Kabab Wala - Queen'!$A:$A, B75, 'Karachi Kabab Wala - Queen'!$F:$F), 0)</f>
         <v/>
       </c>
-      <c r="X75" s="10" t="n"/>
+      <c r="AB75" s="10" t="n"/>
     </row>
     <row r="76">
       <c r="A76" s="55" t="n"/>
@@ -5408,18 +6170,18 @@
       <c r="P76" s="9" t="n"/>
       <c r="Q76" s="9" t="n"/>
       <c r="R76" s="9" t="n"/>
-      <c r="S76" s="9" t="n"/>
-      <c r="T76" s="9" t="n"/>
-      <c r="U76" s="9">
+      <c r="W76" s="9" t="n"/>
+      <c r="X76" s="9" t="n"/>
+      <c r="Y76" s="9">
         <f>IFERROR(SUMIF('Karachi Kabab Wala'!$A:$A, B76, 'Karachi Kabab Wala'!$F:$F), 0)</f>
         <v/>
       </c>
-      <c r="V76" s="10" t="n"/>
-      <c r="W76" s="9">
+      <c r="Z76" s="10" t="n"/>
+      <c r="AA76" s="9">
         <f>IFERROR(SUMIF('Karachi Kabab Wala - Queen'!$A:$A, B76, 'Karachi Kabab Wala - Queen'!$F:$F), 0)</f>
         <v/>
       </c>
-      <c r="X76" s="10" t="n"/>
+      <c r="AB76" s="10" t="n"/>
     </row>
     <row r="77">
       <c r="A77" s="55" t="n"/>
@@ -5452,22 +6214,22 @@
         </is>
       </c>
       <c r="R77" s="9" t="n"/>
-      <c r="S77" s="9" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="T77" s="9" t="n"/>
-      <c r="U77" s="9">
+      <c r="W77" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="X77" s="9" t="n"/>
+      <c r="Y77" s="9">
         <f>IFERROR(SUMIF('Karachi Kabab Wala'!$A:$A, B77, 'Karachi Kabab Wala'!$F:$F), 0)</f>
         <v/>
       </c>
-      <c r="V77" s="10" t="n"/>
-      <c r="W77" s="9">
+      <c r="Z77" s="10" t="n"/>
+      <c r="AA77" s="9">
         <f>IFERROR(SUMIF('Karachi Kabab Wala - Queen'!$A:$A, B77, 'Karachi Kabab Wala - Queen'!$F:$F), 0)</f>
         <v/>
       </c>
-      <c r="X77" s="10" t="n"/>
+      <c r="AB77" s="10" t="n"/>
     </row>
     <row r="78">
       <c r="A78" s="56" t="n"/>
@@ -5524,22 +6286,34 @@
         </is>
       </c>
       <c r="R78" s="26" t="n"/>
-      <c r="S78" s="26" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="T78" s="26" t="n"/>
-      <c r="U78" s="26">
+      <c r="S78" s="60" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="T78" s="60" t="n"/>
+      <c r="U78" s="60" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="V78" s="60" t="n"/>
+      <c r="W78" s="26" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="X78" s="26" t="n"/>
+      <c r="Y78" s="26">
         <f>IFERROR(SUMIF('Karachi Kabab Wala'!$A:$A, B78, 'Karachi Kabab Wala'!$F:$F), 0)</f>
         <v/>
       </c>
-      <c r="V78" s="29" t="n"/>
-      <c r="W78" s="26">
+      <c r="Z78" s="29" t="n"/>
+      <c r="AA78" s="26">
         <f>IFERROR(SUMIF('Karachi Kabab Wala - Queen'!$A:$A, B78, 'Karachi Kabab Wala - Queen'!$F:$F), 0)</f>
         <v/>
       </c>
-      <c r="X78" s="29" t="n"/>
+      <c r="AB78" s="29" t="n"/>
     </row>
     <row r="79" ht="15" customHeight="1">
       <c r="A79" s="57" t="inlineStr">
@@ -5599,22 +6373,34 @@
         </is>
       </c>
       <c r="R79" s="15" t="n"/>
-      <c r="S79" s="15" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="T79" s="15" t="n"/>
-      <c r="U79" s="15">
+      <c r="S79" s="59" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="T79" s="59" t="n"/>
+      <c r="U79" s="59" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="V79" s="59" t="n"/>
+      <c r="W79" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="X79" s="15" t="n"/>
+      <c r="Y79" s="15">
         <f>IFERROR(SUMIF('Karachi Kabab Wala'!$A:$A, B79, 'Karachi Kabab Wala'!$F:$F), 0)</f>
         <v/>
       </c>
-      <c r="V79" s="15" t="n"/>
-      <c r="W79" s="15">
+      <c r="Z79" s="15" t="n"/>
+      <c r="AA79" s="15">
         <f>IFERROR(SUMIF('Karachi Kabab Wala - Queen'!$A:$A, B79, 'Karachi Kabab Wala - Queen'!$F:$F), 0)</f>
         <v/>
       </c>
-      <c r="X79" s="23" t="n"/>
+      <c r="AB79" s="23" t="n"/>
     </row>
     <row r="80" ht="15" customHeight="1">
       <c r="B80" s="30" t="inlineStr">
@@ -5669,22 +6455,34 @@
         </is>
       </c>
       <c r="R80" s="15" t="n"/>
-      <c r="S80" s="15" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="T80" s="15" t="n"/>
-      <c r="U80" s="15">
+      <c r="S80" s="59" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="T80" s="59" t="n"/>
+      <c r="U80" s="59" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="V80" s="59" t="n"/>
+      <c r="W80" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="X80" s="15" t="n"/>
+      <c r="Y80" s="15">
         <f>IFERROR(SUMIF('Karachi Kabab Wala'!$A:$A, B80, 'Karachi Kabab Wala'!$F:$F), 0)</f>
         <v/>
       </c>
-      <c r="V80" s="15" t="n"/>
-      <c r="W80" s="15">
+      <c r="Z80" s="15" t="n"/>
+      <c r="AA80" s="15">
         <f>IFERROR(SUMIF('Karachi Kabab Wala - Queen'!$A:$A, B80, 'Karachi Kabab Wala - Queen'!$F:$F), 0)</f>
         <v/>
       </c>
-      <c r="X80" s="23" t="n"/>
+      <c r="AB80" s="23" t="n"/>
     </row>
     <row r="81" ht="15" customHeight="1">
       <c r="B81" s="32" t="inlineStr">
@@ -5711,12 +6509,12 @@
       <c r="P81" s="15" t="n"/>
       <c r="Q81" s="15" t="n"/>
       <c r="R81" s="15" t="n"/>
-      <c r="S81" s="15" t="n"/>
-      <c r="T81" s="15" t="n"/>
-      <c r="U81" s="15" t="n"/>
-      <c r="V81" s="15" t="n"/>
-      <c r="W81" s="23" t="n"/>
-      <c r="X81" s="23" t="n"/>
+      <c r="W81" s="15" t="n"/>
+      <c r="X81" s="15" t="n"/>
+      <c r="Y81" s="15" t="n"/>
+      <c r="Z81" s="15" t="n"/>
+      <c r="AA81" s="23" t="n"/>
+      <c r="AB81" s="23" t="n"/>
     </row>
     <row r="82" ht="15" customHeight="1" thickBot="1">
       <c r="A82" s="44" t="n"/>
@@ -5744,12 +6542,12 @@
       <c r="P82" s="18" t="n"/>
       <c r="Q82" s="18" t="n"/>
       <c r="R82" s="18" t="n"/>
-      <c r="S82" s="18" t="n"/>
-      <c r="T82" s="18" t="n"/>
-      <c r="U82" s="18" t="n"/>
-      <c r="V82" s="18" t="n"/>
-      <c r="W82" s="35" t="n"/>
-      <c r="X82" s="35" t="n"/>
+      <c r="W82" s="18" t="n"/>
+      <c r="X82" s="18" t="n"/>
+      <c r="Y82" s="18" t="n"/>
+      <c r="Z82" s="18" t="n"/>
+      <c r="AA82" s="35" t="n"/>
+      <c r="AB82" s="35" t="n"/>
     </row>
     <row r="83" ht="14.45" customHeight="1"/>
   </sheetData>
@@ -5758,7 +6556,7 @@
     <mergeCell ref="A79:A82"/>
     <mergeCell ref="A46:A58"/>
     <mergeCell ref="A59:A78"/>
-    <mergeCell ref="A1:X2"/>
+    <mergeCell ref="A1:AB2"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B10" display="https://admin.touchbistro.com/venue-management/bases/01439546-d97c-445a-8cb5-be2395ed6522/menu-management/menu-items/df6f390b-46a4-4b51-89f5-1516c0211b2d/edit" r:id="rId1"/>

</xml_diff>